<commit_message>
feat: SimSeries/SimDataFrame/SimBasics class hierarchy foundation
</commit_message>
<xml_diff>
--- a/test/_testing_data/dimensions.xlsx
+++ b/test/_testing_data/dimensions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\simpandas\test\_testing_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F729C95-E518-45CE-BEE4-604CFC09F57D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F8E07C-FCEC-4D70-8D7F-7803FC5B7AA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="40" windowWidth="19750" windowHeight="20410" xr2:uid="{03D7C936-FFF9-42D8-9C7E-DA00DB89D8CB}"/>
+    <workbookView xWindow="11750" yWindow="1650" windowWidth="24630" windowHeight="18100" xr2:uid="{03D7C936-FFF9-42D8-9C7E-DA00DB89D8CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>item</t>
   </si>
@@ -55,13 +55,22 @@
     <t>wide</t>
   </si>
   <si>
-    <t>tv</t>
-  </si>
-  <si>
     <t>diagonal</t>
   </si>
   <si>
     <t>in</t>
+  </si>
+  <si>
+    <t>TV</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>heigth</t>
+  </si>
+  <si>
+    <t>um</t>
   </si>
 </sst>
 </file>
@@ -413,10 +422,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78831B2A-CB20-4433-B9B4-806CA708DE34}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -427,21 +436,27 @@
         <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -449,10 +464,13 @@
         <v>15</v>
       </c>
       <c r="C3">
-        <v>0.5</v>
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>5000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -460,14 +478,17 @@
         <v>29.7</v>
       </c>
       <c r="C4">
-        <v>21.1</v>
+        <v>210</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
         <v>65</v>
       </c>
     </row>

</xml_diff>